<commit_message>
Pass F4 reconstruct full extracted spec fields
</commit_message>
<xml_diff>
--- a/data/synthetic/rendered/oem_b.xlsx
+++ b/data/synthetic/rendered/oem_b.xlsx
@@ -847,7 +847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -878,6 +878,21 @@
           <t>Parameter octets</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Allowed modes</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Access tier</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -900,6 +915,21 @@
           <t>{'1': 2, '2': 0}</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -922,6 +952,21 @@
           <t>{'1': 2, '2': 0}</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -944,10 +989,25 @@
           <t>{'1': 2, '2': 0}</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -959,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -990,6 +1050,16 @@
           <t>Security gate</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Subfunctions</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SPR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1003,6 +1073,19 @@
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1016,6 +1099,19 @@
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>[{'value': 1, 'name': 'hard'}]</t>
+        </is>
+      </c>
+      <c r="F4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1029,6 +1125,19 @@
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1042,6 +1151,19 @@
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1055,6 +1177,19 @@
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1072,8 +1207,18 @@
           <t>4</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>2</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1088,10 +1233,23 @@
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1193,7 +1351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1206,14 +1364,126 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>The six operating conditions are ignition_on, speed_zero, doors_closed, battery_ok, vehicle_stopped, and service_brake.</t>
+          <t>DID 0x2000 may be written only when ignition_on is true.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Each condition must be true for its matching data identifier write.</t>
+          <t>Writing DID 0x2000 requires ignition_on to be true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DID 0x2000 must not be written while ignition_on is false.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DID 0x2001 may be written only when speed_zero is true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Writing DID 0x2001 requires speed_zero to be true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DID 0x2001 must not be written while speed_zero is false.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DID 0x2002 may be written only when doors_closed is true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Writing DID 0x2002 requires doors_closed to be true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DID 0x2002 must not be written while doors_closed is false.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DID 0x2003 may be written only when battery_ok is true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Writing DID 0x2003 requires battery_ok to be true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DID 0x2003 must not be written while battery_ok is false.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>DID 0x2004 may be written only when vehicle_stopped is true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Writing DID 0x2004 requires vehicle_stopped to be true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>DID 0x2004 must not be written while vehicle_stopped is false.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DID 0x2005 may be written only when service_brake is true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Writing DID 0x2005 requires service_brake to be true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DID 0x2005 must not be written while service_brake is false.</t>
         </is>
       </c>
     </row>

</xml_diff>